<commit_message>
error log for spring25 rx
</commit_message>
<xml_diff>
--- a/Error Logs/ThunderMountain_2026.xlsx
+++ b/Error Logs/ThunderMountain_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/cfossum_nps_gov1/Documents/Desktop/FFI_QAQC/Error Logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_E116DCD0B0C9EF856C2653374BD29FCC71F0A0AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D3011DF-7096-4F06-B334-89DAC2DCE25F}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_E116DCD0B0C9EF856C2653374BD29FCC71F0A0AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4832BBCB-F9EB-4D54-AEAB-D2FBB5B253DF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -571,7 +571,7 @@
     <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="62.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>